<commit_message>
added week 2 day-2
</commit_message>
<xml_diff>
--- a/DE_GenAI_Intern_Training_3Weeks.xlsx
+++ b/DE_GenAI_Intern_Training_3Weeks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\om\Desktop\AI-GenAI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B570C5E6-3613-44FE-8FFD-C40175A7741B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{340CBEC7-4F38-4287-916F-E1A8FA6C2582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -1555,29 +1555,11 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1589,14 +1571,32 @@
     <xf numFmtId="0" fontId="11" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1843,7 +1843,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="46" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="28"/>
@@ -1854,7 +1854,7 @@
       <c r="H2" s="29"/>
     </row>
     <row r="3" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="47" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="28"/>
@@ -1865,7 +1865,7 @@
       <c r="H3" s="29"/>
     </row>
     <row r="5" spans="2:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="40" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="28"/>
@@ -1876,11 +1876,11 @@
       <c r="H5" s="29"/>
     </row>
     <row r="6" spans="2:8" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="43" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="29"/>
-      <c r="D6" s="37" t="s">
+      <c r="D6" s="44" t="s">
         <v>4</v>
       </c>
       <c r="E6" s="28"/>
@@ -1889,11 +1889,11 @@
       <c r="H6" s="29"/>
     </row>
     <row r="7" spans="2:8" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="41" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="29"/>
-      <c r="D7" s="39" t="s">
+      <c r="D7" s="42" t="s">
         <v>6</v>
       </c>
       <c r="E7" s="28"/>
@@ -1902,11 +1902,11 @@
       <c r="H7" s="29"/>
     </row>
     <row r="8" spans="2:8" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="36" t="s">
+      <c r="B8" s="43" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="29"/>
-      <c r="D8" s="37" t="s">
+      <c r="D8" s="44" t="s">
         <v>8</v>
       </c>
       <c r="E8" s="28"/>
@@ -1915,7 +1915,7 @@
       <c r="H8" s="29"/>
     </row>
     <row r="10" spans="2:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="40" t="s">
+      <c r="B10" s="45" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="28"/>
@@ -1932,15 +1932,15 @@
       <c r="C11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="41" t="s">
+      <c r="D11" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="42"/>
-      <c r="F11" s="41" t="s">
+      <c r="E11" s="36"/>
+      <c r="F11" s="35" t="s">
         <v>13</v>
       </c>
       <c r="G11" s="31"/>
-      <c r="H11" s="42"/>
+      <c r="H11" s="36"/>
     </row>
     <row r="12" spans="2:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="2" t="s">
@@ -1949,11 +1949,11 @@
       <c r="C12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="43" t="s">
+      <c r="D12" s="37" t="s">
         <v>16</v>
       </c>
       <c r="E12" s="32"/>
-      <c r="F12" s="44" t="s">
+      <c r="F12" s="38" t="s">
         <v>17</v>
       </c>
       <c r="G12" s="31"/>
@@ -1966,11 +1966,11 @@
       <c r="C13" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="46" t="s">
+      <c r="D13" s="39" t="s">
         <v>20</v>
       </c>
       <c r="E13" s="32"/>
-      <c r="F13" s="45" t="s">
+      <c r="F13" s="34" t="s">
         <v>21</v>
       </c>
       <c r="G13" s="31"/>
@@ -1983,18 +1983,18 @@
       <c r="C14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="43" t="s">
+      <c r="D14" s="37" t="s">
         <v>24</v>
       </c>
       <c r="E14" s="32"/>
-      <c r="F14" s="44" t="s">
+      <c r="F14" s="38" t="s">
         <v>25</v>
       </c>
       <c r="G14" s="31"/>
       <c r="H14" s="32"/>
     </row>
     <row r="16" spans="2:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="35" t="s">
+      <c r="B16" s="40" t="s">
         <v>26</v>
       </c>
       <c r="C16" s="28"/>
@@ -2008,20 +2008,20 @@
       <c r="B17" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="41" t="s">
+      <c r="C17" s="35" t="s">
         <v>28</v>
       </c>
       <c r="D17" s="31"/>
       <c r="E17" s="31"/>
       <c r="F17" s="31"/>
       <c r="G17" s="31"/>
-      <c r="H17" s="42"/>
+      <c r="H17" s="36"/>
     </row>
     <row r="18" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="47" t="s">
+      <c r="C18" s="33" t="s">
         <v>30</v>
       </c>
       <c r="D18" s="31"/>
@@ -2034,7 +2034,7 @@
       <c r="B19" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="45" t="s">
+      <c r="C19" s="34" t="s">
         <v>32</v>
       </c>
       <c r="D19" s="31"/>
@@ -2047,7 +2047,7 @@
       <c r="B20" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="47" t="s">
+      <c r="C20" s="33" t="s">
         <v>34</v>
       </c>
       <c r="D20" s="31"/>
@@ -2060,7 +2060,7 @@
       <c r="B21" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="45" t="s">
+      <c r="C21" s="34" t="s">
         <v>36</v>
       </c>
       <c r="D21" s="31"/>
@@ -2073,7 +2073,7 @@
       <c r="B22" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C22" s="47" t="s">
+      <c r="C22" s="33" t="s">
         <v>38</v>
       </c>
       <c r="D22" s="31"/>
@@ -2086,7 +2086,7 @@
       <c r="B23" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="45" t="s">
+      <c r="C23" s="34" t="s">
         <v>40</v>
       </c>
       <c r="D23" s="31"/>
@@ -2099,7 +2099,7 @@
       <c r="B24" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C24" s="47" t="s">
+      <c r="C24" s="33" t="s">
         <v>42</v>
       </c>
       <c r="D24" s="31"/>
@@ -3086,11 +3086,16 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="C20:H20"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
-    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="B10:H10"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="F11:H11"/>
     <mergeCell ref="D12:E12"/>
@@ -3103,16 +3108,11 @@
     <mergeCell ref="B16:H16"/>
     <mergeCell ref="C17:H17"/>
     <mergeCell ref="C18:H18"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="C20:H20"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
+    <mergeCell ref="C24:H24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -8308,7 +8308,7 @@
       <c r="E4" s="32"/>
     </row>
     <row r="5" spans="2:5" ht="129.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="45" t="s">
+      <c r="B5" s="34" t="s">
         <v>278</v>
       </c>
       <c r="C5" s="32"/>
@@ -8328,7 +8328,7 @@
       <c r="E7" s="32"/>
     </row>
     <row r="8" spans="2:5" ht="129.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="45" t="s">
+      <c r="B8" s="34" t="s">
         <v>282</v>
       </c>
       <c r="C8" s="32"/>
@@ -8348,7 +8348,7 @@
       <c r="E10" s="32"/>
     </row>
     <row r="11" spans="2:5" ht="129.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="45" t="s">
+      <c r="B11" s="34" t="s">
         <v>286</v>
       </c>
       <c r="C11" s="32"/>

</xml_diff>